<commit_message>
Switch RX-8 route to self-made adapter plate and CSC adapter
Bought plate/bolts/CSC kit are now off by default; material lines for
the self-machined parts added. Note that CEED's lasers are CO2 only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0175jEiqU2oBgc19VRi9yMgm
</commit_message>
<xml_diff>
--- a/Gearbox_Options.xlsx
+++ b/Gearbox_Options.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="214">
   <si>
     <t xml:space="preserve">07K gearbox options: RX-8 6-speed manual vs ZF 8HP automatic</t>
   </si>
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Adapter</t>
   </si>
   <si>
-    <t xml:space="preserve">£140 plate + £35 bolts + £10 spigot from one UK shop; in stock, ships next day.</t>
+    <t xml:space="preserve">Make your own at Brunsfield (material ~US$150–300), or buy the proven £140 plate + £35 bolts from RX8 Gearbox Adapters.</t>
   </si>
   <si>
     <t xml:space="preserve">$1,250–1,280 DomiWorks kit (plate + billet flywheel + centre guide). Also sold by a Quebec dealer.</t>
@@ -97,7 +97,7 @@
     <t xml:space="preserve">Clutch / release</t>
   </si>
   <si>
-    <t xml:space="preserve">Concentric slave kit £230 (fork is blocked by the 07K casting). Needs careful spacer setup.</t>
+    <t xml:space="preserve">Concentric slave (fork is blocked by the 07K casting): make the adapter + spacers, buy the slave unit. Needs careful spacer setup.</t>
   </si>
   <si>
     <t xml:space="preserve">None (auto).</t>
@@ -241,12 +241,15 @@
     <t xml:space="preserve">Adapter plate: VW PD/1.8T 20V → RX-8, upright (RX8002)</t>
   </si>
   <si>
-    <t xml:space="preserve">Engine sits upright instead of VW's 15° lean. Usually in stock, ships next working day. Brett Horn's first-video plate — his build needed a 'resolving bolt alignment' step, so confirm the 07K holes line up.</t>
+    <t xml:space="preserve">Engine sits upright instead of VW's 15° lean. Usually in stock, ships next working day. Brett Horn's first-video plate — his build needed a 'resolving bolt alignment' step, so confirm the 07K holes line up. OFF by default: you are making your own (R3M).</t>
   </si>
   <si>
     <t xml:space="preserve">GBP</t>
   </si>
   <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.rx8gearboxadapters.com/product-page/vw-pd-1-8t-20v-vertically-mounted</t>
   </si>
   <si>
@@ -259,9 +262,6 @@
     <t xml:space="preserve">Made to order (~2 weeks). Brett switched to this one to tilt the engine for clearance. Set Include = Y and R3 = N to switch.</t>
   </si>
   <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.rx8gearboxadapters.com/product-page/copy-of-vw-pd-1-8t-20v-mounted-20degrees</t>
   </si>
   <si>
@@ -271,7 +271,7 @@
     <t xml:space="preserve">Bolt kit (RX8027)</t>
   </si>
   <si>
-    <t xml:space="preserve">High-tensile cap heads + nylocs: plate→block and RX-8 bell→plate.</t>
+    <t xml:space="preserve">High-tensile cap heads + nylocs: plate→block and RX-8 bell→plate. OFF by default: lengths depend on your plate thickness (see R5M).</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.rx8gearboxadapters.com/product-page/vw-pd-1-8t-bolt-kit-rx8027</t>
@@ -295,7 +295,7 @@
     <t xml:space="preserve">Concentric slave cylinder kit, RX-8 6-speed (RX8032)</t>
   </si>
   <si>
-    <t xml:space="preserve">CSC (42 mm ID / 63 mm OD bearing), billet adapter, spacer plates, hardware, PDF setup guide. Brett needed a CSC because the 07K timing-cover / vacuum-pump casting blocks the RX-8 fork. Set N to try the stock RX-8 slave + fork first.</t>
+    <t xml:space="preserve">CSC (42 mm ID / 63 mm OD bearing), billet adapter, spacer plates, hardware, PDF setup guide. Brett needed a CSC because the 07K timing-cover / vacuum-pump casting blocks the RX-8 fork. Set N to try the stock RX-8 slave + fork first. OFF by default: making the adapter + spacers yourself (R7M–R7M3) — but note the slave unit alone can cost more than this whole kit.</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.rx8gearboxadapters.com/product-page/rx8-6-speed-concentric-slave-cylinder-set-up</t>
@@ -304,15 +304,78 @@
     <t xml:space="preserve">R8</t>
   </si>
   <si>
-    <t xml:space="preserve">UK → Canada courier for the adapter parts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rough courier cost. UK-origin parts are duty-free under the Canada–UK trade agreement; HST is charged on the Summary tab.</t>
+    <t xml:space="preserve">UK → Canada courier (spigot bearing only now)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rough courier cost; or find the same bearing size locally. UK-origin parts are duty-free under the Canada–UK trade agreement; HST is charged on the Summary tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Estimate</t>
   </si>
   <si>
+    <t xml:space="preserve">R3M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAKE: adapter plate — 6061-T6 (or MIC-6 cast) plate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~16 × 16 in blank; thickness from your stack-up (§13). Machine at Brunsfield: profile, bolt holes, starter mount, dowel holes drilled + reamed. CEED's CO2 lasers can't cut aluminium; SendCutSend can laser it (≤0.75 in, ±0.005 in) if there's no CNC. 1/4 in × 16 × 16 is ~US$67, so 3/4 in is roughly 3×.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ebay.com/itm/365068559418</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R3M2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAKE: dowel pins (hardened) + reamer if the shop lacks the size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Match the VW block and RX-8 bell dowel diameters. Add offset dowels if runout &gt; 0.005 in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://americanpowertrain.com/general-bellhousing-alignment-instructions/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R5M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAKE: fasteners — 10.9 cap screws, nuts, washers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Block→plate and bell→plate; lengths from your plate thickness.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R7M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUY: concentric slave cylinder unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The only part of the slave setup you can't make. Range: a cheap OE-style CSC (if you find one whose bore clears the RX-8 snout) up to a Tilton 1000/6100-series universal (US$370–460).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.speedwaymotors.com/Tilton-60-6100-Flat-Face-Hydraulic-Release-Bearing-Universal,413901.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R7M2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAKE: CSC mounting adapter — 6061 round bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~4–5 in dia × 2 in. Lathe part: bore over the RX-8 input snout, M8 pattern to the box, M6 pattern for the CSC.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R7M3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAKE: CSC spacer plates — aluminium sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set release-bearing-to-finger gap. Several thicknesses.</t>
+  </si>
+  <si>
     <t xml:space="preserve">R9</t>
   </si>
   <si>
@@ -361,10 +424,10 @@
     <t xml:space="preserve">R13</t>
   </si>
   <si>
-    <t xml:space="preserve">Vacuum pump block-off plate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gives clearance at the bellhousing — the casting still sticks out after the delete (Brett).</t>
+    <t xml:space="preserve">MAKE: vacuum pump block-off plate (only if the pump hits)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aluminium scrap/plate + O-ring, milled at Brunsfield. Only needed if you delete the pump for clearance.</t>
   </si>
   <si>
     <t xml:space="preserve">R14</t>
@@ -1192,8 +1255,8 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">'RX-8 BOM'!H22</f>
-        <v>2893.1955</v>
+        <f aca="false">'RX-8 BOM'!H28</f>
+        <v>2475.6605</v>
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">'8HP BOM'!H23</f>
@@ -1205,8 +1268,8 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">'RX-8 BOM'!I22</f>
-        <v>5375.8846</v>
+        <f aca="false">'RX-8 BOM'!I28</f>
+        <v>5925.0081</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">'8HP BOM'!I23</f>
@@ -1220,7 +1283,7 @@
       <c r="B7" s="5"/>
       <c r="C7" s="7" t="n">
         <f aca="false">IF(B5+B6=0,0,(C5+C6)/(B5+B6))</f>
-        <v>2.43666308178585</v>
+        <v>2.39849506740452</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1395,7 +1458,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1574,7 +1637,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
         <v>70</v>
       </c>
@@ -1598,31 +1661,31 @@
       </c>
       <c r="H7" s="17" t="n">
         <f aca="false">IF($J7="Y",$D7*$F7*INDEX(Assumptions!$B$4:$B$6,MATCH($E7,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>259</v>
+        <v>0</v>
       </c>
       <c r="I7" s="17" t="n">
         <f aca="false">IF($J7="Y",$D7*$G7*INDEX(Assumptions!$B$4:$B$6,MATCH($E7,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>259</v>
+        <v>0</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="K7" s="13" t="s">
         <v>65</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>1</v>
@@ -1645,7 +1708,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>65</v>
@@ -1654,7 +1717,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
         <v>80</v>
       </c>
@@ -1678,14 +1741,14 @@
       </c>
       <c r="H9" s="17" t="n">
         <f aca="false">IF($J9="Y",$D9*$F9*INDEX(Assumptions!$B$4:$B$6,MATCH($E9,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>64.75</v>
+        <v>0</v>
       </c>
       <c r="I9" s="17" t="n">
         <f aca="false">IF($J9="Y",$D9*$G9*INDEX(Assumptions!$B$4:$B$6,MATCH($E9,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>64.75</v>
+        <v>0</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="K9" s="13" t="s">
         <v>65</v>
@@ -1734,7 +1797,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
         <v>88</v>
       </c>
@@ -1758,14 +1821,14 @@
       </c>
       <c r="H11" s="17" t="n">
         <f aca="false">IF($J11="Y",$D11*$F11*INDEX(Assumptions!$B$4:$B$6,MATCH($E11,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>425.5</v>
+        <v>0</v>
       </c>
       <c r="I11" s="17" t="n">
         <f aca="false">IF($J11="Y",$D11*$G11*INDEX(Assumptions!$B$4:$B$6,MATCH($E11,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>425.5</v>
+        <v>0</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="K11" s="13" t="s">
         <v>65</v>
@@ -1791,18 +1854,18 @@
         <v>73</v>
       </c>
       <c r="F12" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" s="16" t="n">
         <v>40</v>
-      </c>
-      <c r="G12" s="16" t="n">
-        <v>90</v>
       </c>
       <c r="H12" s="17" t="n">
         <f aca="false">IF($J12="Y",$D12*$F12*INDEX(Assumptions!$B$4:$B$6,MATCH($E12,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>74</v>
+        <v>27.75</v>
       </c>
       <c r="I12" s="17" t="n">
         <f aca="false">IF($J12="Y",$D12*$G12*INDEX(Assumptions!$B$4:$B$6,MATCH($E12,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>166.5</v>
+        <v>74</v>
       </c>
       <c r="J12" s="15" t="s">
         <v>64</v>
@@ -1829,24 +1892,24 @@
         <v>63</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>400</v>
+        <v>150</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>726</v>
+        <v>300</v>
       </c>
       <c r="H13" s="17" t="n">
         <f aca="false">IF($J13="Y",$D13*$F13*INDEX(Assumptions!$B$4:$B$6,MATCH($E13,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>568</v>
+        <v>213</v>
       </c>
       <c r="I13" s="17" t="n">
         <f aca="false">IF($J13="Y",$D13*$G13*INDEX(Assumptions!$B$4:$B$6,MATCH($E13,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>1030.92</v>
+        <v>426</v>
       </c>
       <c r="J13" s="15" t="s">
         <v>64</v>
       </c>
       <c r="K13" s="13" t="s">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="L13" s="18" t="s">
         <v>99</v>
@@ -1866,21 +1929,21 @@
         <v>1</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="H14" s="17" t="n">
         <f aca="false">IF($J14="Y",$D14*$F14*INDEX(Assumptions!$B$4:$B$6,MATCH($E14,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>111</v>
+        <v>42.6</v>
       </c>
       <c r="I14" s="17" t="n">
         <f aca="false">IF($J14="Y",$D14*$G14*INDEX(Assumptions!$B$4:$B$6,MATCH($E14,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>277.5</v>
+        <v>127.8</v>
       </c>
       <c r="J14" s="15" t="s">
         <v>64</v>
@@ -1892,7 +1955,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
         <v>104</v>
       </c>
@@ -1906,41 +1969,39 @@
         <v>1</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="F15" s="16" t="n">
         <v>40</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>145</v>
+        <v>80</v>
       </c>
       <c r="H15" s="17" t="n">
         <f aca="false">IF($J15="Y",$D15*$F15*INDEX(Assumptions!$B$4:$B$6,MATCH($E15,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>74</v>
+        <v>56.8</v>
       </c>
       <c r="I15" s="17" t="n">
         <f aca="false">IF($J15="Y",$D15*$G15*INDEX(Assumptions!$B$4:$B$6,MATCH($E15,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>268.25</v>
+        <v>113.6</v>
       </c>
       <c r="J15" s="15" t="s">
         <v>64</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="L15" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="L15" s="14"/>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="B16" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="C16" s="14" t="s">
         <v>109</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>110</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>1</v>
@@ -1949,18 +2010,18 @@
         <v>63</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>100</v>
+        <v>460</v>
       </c>
       <c r="H16" s="17" t="n">
         <f aca="false">IF($J16="Y",$D16*$F16*INDEX(Assumptions!$B$4:$B$6,MATCH($E16,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>56.8</v>
+        <v>113.6</v>
       </c>
       <c r="I16" s="17" t="n">
         <f aca="false">IF($J16="Y",$D16*$G16*INDEX(Assumptions!$B$4:$B$6,MATCH($E16,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>142</v>
+        <v>653.2</v>
       </c>
       <c r="J16" s="15" t="s">
         <v>64</v>
@@ -1968,7 +2029,9 @@
       <c r="K16" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="L16" s="14"/>
+      <c r="L16" s="18" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
@@ -1987,18 +2050,18 @@
         <v>63</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="G17" s="16" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="H17" s="17" t="n">
         <f aca="false">IF($J17="Y",$D17*$F17*INDEX(Assumptions!$B$4:$B$6,MATCH($E17,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>56.8</v>
+        <v>42.6</v>
       </c>
       <c r="I17" s="17" t="n">
         <f aca="false">IF($J17="Y",$D17*$G17*INDEX(Assumptions!$B$4:$B$6,MATCH($E17,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>113.6</v>
+        <v>85.2</v>
       </c>
       <c r="J17" s="15" t="s">
         <v>64</v>
@@ -2025,18 +2088,18 @@
         <v>63</v>
       </c>
       <c r="F18" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="16" t="n">
         <v>25</v>
-      </c>
-      <c r="G18" s="16" t="n">
-        <v>50</v>
       </c>
       <c r="H18" s="17" t="n">
         <f aca="false">IF($J18="Y",$D18*$F18*INDEX(Assumptions!$B$4:$B$6,MATCH($E18,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>35.5</v>
+        <v>14.2</v>
       </c>
       <c r="I18" s="17" t="n">
         <f aca="false">IF($J18="Y",$D18*$G18*INDEX(Assumptions!$B$4:$B$6,MATCH($E18,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>71</v>
+        <v>35.5</v>
       </c>
       <c r="J18" s="15" t="s">
         <v>64</v>
@@ -2046,7 +2109,7 @@
       </c>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
         <v>117</v>
       </c>
@@ -2060,108 +2123,342 @@
         <v>1</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="G19" s="16" t="n">
-        <v>10</v>
+        <v>726</v>
       </c>
       <c r="H19" s="17" t="n">
         <f aca="false">IF($J19="Y",$D19*$F19*INDEX(Assumptions!$B$4:$B$6,MATCH($E19,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>0</v>
+        <v>568</v>
       </c>
       <c r="I19" s="17" t="n">
         <f aca="false">IF($J19="Y",$D19*$G19*INDEX(Assumptions!$B$4:$B$6,MATCH($E19,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>10</v>
+        <v>1030.92</v>
       </c>
       <c r="J19" s="15" t="s">
         <v>64</v>
       </c>
       <c r="K19" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L19" s="18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="F20" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="G20" s="16" t="n">
+        <v>150</v>
+      </c>
+      <c r="H20" s="17" t="n">
+        <f aca="false">IF($J20="Y",$D20*$F20*INDEX(Assumptions!$B$4:$B$6,MATCH($E20,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>111</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <f aca="false">IF($J20="Y",$D20*$G20*INDEX(Assumptions!$B$4:$B$6,MATCH($E20,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>277.5</v>
+      </c>
+      <c r="J20" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="K20" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="L19" s="14"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="H20" s="20" t="n">
-        <f aca="false">SUM(H5:H19)</f>
-        <v>2560.35</v>
-      </c>
-      <c r="I20" s="20" t="n">
-        <f aca="false">SUM(I5:I19)</f>
-        <v>4757.42</v>
-      </c>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="19" t="s">
-        <v>122</v>
-      </c>
-      <c r="H21" s="20" t="n">
-        <f aca="false">H20*Assumptions!$B$8</f>
-        <v>332.8455</v>
-      </c>
-      <c r="I21" s="20" t="n">
-        <f aca="false">I20*Assumptions!$B$8</f>
-        <v>618.4646</v>
-      </c>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
+      <c r="L20" s="18" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>145</v>
+      </c>
+      <c r="H21" s="17" t="n">
+        <f aca="false">IF($J21="Y",$D21*$F21*INDEX(Assumptions!$B$4:$B$6,MATCH($E21,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>74</v>
+      </c>
+      <c r="I21" s="17" t="n">
+        <f aca="false">IF($J21="Y",$D21*$G21*INDEX(Assumptions!$B$4:$B$6,MATCH($E21,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>268.25</v>
+      </c>
+      <c r="J21" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="K21" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="L21" s="18" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="H22" s="22" t="n">
-        <f aca="false">H20+H21</f>
-        <v>2893.1955</v>
-      </c>
-      <c r="I22" s="22" t="n">
-        <f aca="false">I20+I21</f>
-        <v>5375.8846</v>
-      </c>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
+      <c r="A22" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F22" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="G22" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <f aca="false">IF($J22="Y",$D22*$F22*INDEX(Assumptions!$B$4:$B$6,MATCH($E22,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>56.8</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <f aca="false">IF($J22="Y",$D22*$G22*INDEX(Assumptions!$B$4:$B$6,MATCH($E22,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>142</v>
+      </c>
+      <c r="J22" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="L22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G23" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="H23" s="17" t="n">
+        <f aca="false">IF($J23="Y",$D23*$F23*INDEX(Assumptions!$B$4:$B$6,MATCH($E23,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="17" t="n">
+        <f aca="false">IF($J23="Y",$D23*$G23*INDEX(Assumptions!$B$4:$B$6,MATCH($E23,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="K23" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="L23" s="14"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="G24" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <f aca="false">IF($J24="Y",$D24*$F24*INDEX(Assumptions!$B$4:$B$6,MATCH($E24,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>35.5</v>
+      </c>
+      <c r="I24" s="17" t="n">
+        <f aca="false">IF($J24="Y",$D24*$G24*INDEX(Assumptions!$B$4:$B$6,MATCH($E24,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>71</v>
+      </c>
+      <c r="J24" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="L24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="H25" s="17" t="n">
+        <f aca="false">IF($J25="Y",$D25*$F25*INDEX(Assumptions!$B$4:$B$6,MATCH($E25,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="17" t="n">
+        <f aca="false">IF($J25="Y",$D25*$G25*INDEX(Assumptions!$B$4:$B$6,MATCH($E25,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>10</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="K25" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="L25" s="14"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="H26" s="20" t="n">
+        <f aca="false">SUM(H5:H25)</f>
+        <v>2190.85</v>
+      </c>
+      <c r="I26" s="20" t="n">
+        <f aca="false">SUM(I5:I25)</f>
+        <v>5243.37</v>
+      </c>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="H27" s="20" t="n">
+        <f aca="false">H26*Assumptions!$B$8</f>
+        <v>284.8105</v>
+      </c>
+      <c r="I27" s="20" t="n">
+        <f aca="false">I26*Assumptions!$B$8</f>
+        <v>681.6381</v>
+      </c>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="L27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="H28" s="22" t="n">
+        <f aca="false">H26+H27</f>
+        <v>2475.6605</v>
+      </c>
+      <c r="I28" s="22" t="n">
+        <f aca="false">I26+I27</f>
+        <v>5925.0081</v>
+      </c>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:K19">
+  <conditionalFormatting sqref="A5:K25">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$J5="N"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J19" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J25" type="list">
       <formula1>"Y,N"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E19" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E25" type="list">
       <formula1>"CAD,USD,GBP"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2174,9 +2471,12 @@
     <hyperlink ref="L9" r:id="rId5" display="https://www.rx8gearboxadapters.com/product-page/vw-pd-1-8t-bolt-kit-rx8027"/>
     <hyperlink ref="L10" r:id="rId6" display="https://www.rx8gearboxadapters.com/product-page/rx8-spigot-bearing-rx8017"/>
     <hyperlink ref="L11" r:id="rId7" display="https://www.rx8gearboxadapters.com/product-page/rx8-6-speed-concentric-slave-cylinder-set-up"/>
-    <hyperlink ref="L13" r:id="rId8" display="https://www.ecstuning.com/b-ecs-parts/ra4-single-mass-flywheel-kit/ecs212321b5kt/"/>
-    <hyperlink ref="L14" r:id="rId9" display="https://qedmotorsport.co.uk/product/clutch-plate-228mm-1-x-23-spline-ford-box-heavy-duty-organic-helix/"/>
-    <hyperlink ref="L15" r:id="rId10" display="https://www.ebay.co.uk/p/1509332173"/>
+    <hyperlink ref="L13" r:id="rId8" display="https://www.ebay.com/itm/365068559418"/>
+    <hyperlink ref="L14" r:id="rId9" display="https://americanpowertrain.com/general-bellhousing-alignment-instructions/"/>
+    <hyperlink ref="L16" r:id="rId10" display="https://www.speedwaymotors.com/Tilton-60-6100-Flat-Face-Hydraulic-Release-Bearing-Universal,413901.html"/>
+    <hyperlink ref="L19" r:id="rId11" display="https://www.ecstuning.com/b-ecs-parts/ra4-single-mass-flywheel-kit/ecs212321b5kt/"/>
+    <hyperlink ref="L20" r:id="rId12" display="https://qedmotorsport.co.uk/product/clutch-plate-228mm-1-x-23-spline-ford-box-heavy-duty-organic-helix/"/>
+    <hyperlink ref="L21" r:id="rId13" display="https://www.ebay.co.uk/p/1509332173"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2210,7 +2510,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2294,13 +2594,13 @@
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="D5" s="15" t="n">
         <v>1</v>
@@ -2329,18 +2629,18 @@
         <v>65</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>1</v>
@@ -2369,18 +2669,18 @@
         <v>95</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="D7" s="15" t="n">
         <v>1</v>
@@ -2409,12 +2709,12 @@
         <v>65</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>68</v>
@@ -2447,18 +2747,18 @@
         <v>65</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>1</v>
@@ -2487,18 +2787,18 @@
         <v>65</v>
       </c>
       <c r="L9" s="18" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>1</v>
@@ -2527,18 +2827,18 @@
         <v>65</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>146</v>
+        <v>167</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>1</v>
@@ -2561,24 +2861,24 @@
         <v>0</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K11" s="13" t="s">
         <v>65</v>
       </c>
       <c r="L11" s="18" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>1</v>
@@ -2601,24 +2901,24 @@
         <v>0</v>
       </c>
       <c r="J12" s="15" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K12" s="13" t="s">
         <v>65</v>
       </c>
       <c r="L12" s="18" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>1</v>
@@ -2647,18 +2947,18 @@
         <v>65</v>
       </c>
       <c r="L13" s="18" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>1</v>
@@ -2681,7 +2981,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="15" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K14" s="13" t="s">
         <v>95</v>
@@ -2690,13 +2990,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="D15" s="15" t="n">
         <v>1</v>
@@ -2725,15 +3025,15 @@
         <v>65</v>
       </c>
       <c r="L15" s="18" t="s">
-        <v>164</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>165</v>
+        <v>186</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="15" t="n">
@@ -2766,13 +3066,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>1</v>
@@ -2801,18 +3101,18 @@
         <v>65</v>
       </c>
       <c r="L17" s="18" t="s">
-        <v>170</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>172</v>
+        <v>193</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="D18" s="15" t="n">
         <v>1</v>
@@ -2841,18 +3141,18 @@
         <v>65</v>
       </c>
       <c r="L18" s="18" t="s">
-        <v>174</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>176</v>
+        <v>197</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="D19" s="15" t="n">
         <v>1</v>
@@ -2884,13 +3184,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>179</v>
+        <v>200</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="D20" s="15" t="n">
         <v>1</v>
@@ -2913,13 +3213,13 @@
         <v>0</v>
       </c>
       <c r="J20" s="15" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K20" s="13" t="s">
         <v>65</v>
       </c>
       <c r="L20" s="18" t="s">
-        <v>181</v>
+        <v>202</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2930,7 +3230,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="19" t="s">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="H21" s="20" t="n">
         <f aca="false">SUM(H5:H20)</f>
@@ -2952,7 +3252,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="19" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="H22" s="20" t="n">
         <f aca="false">H21*Assumptions!$B$8</f>
@@ -2974,7 +3274,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="21" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="H23" s="22" t="n">
         <f aca="false">H21+H22</f>
@@ -3044,7 +3344,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>182</v>
+        <v>203</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3056,10 +3356,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>184</v>
+        <v>205</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>59</v>
@@ -3067,13 +3367,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="B4" s="23" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>185</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3084,7 +3384,7 @@
         <v>1.42</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>186</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3095,7 +3395,7 @@
         <v>1.85</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>187</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3105,13 +3405,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="B8" s="25" t="n">
         <v>0.13</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3121,21 +3421,21 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>

</xml_diff>

<commit_message>
Add paid machine-shop labour to the RX-8 make route
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0175jEiqU2oBgc19VRi9yMgm
</commit_message>
<xml_diff>
--- a/Gearbox_Options.xlsx
+++ b/Gearbox_Options.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="217">
   <si>
     <t xml:space="preserve">07K gearbox options: RX-8 6-speed manual vs ZF 8HP automatic</t>
   </si>
@@ -319,7 +319,7 @@
     <t xml:space="preserve">MAKE: adapter plate — 6061-T6 (or MIC-6 cast) plate</t>
   </si>
   <si>
-    <t xml:space="preserve">~16 × 16 in blank; thickness from your stack-up (§13). Machine at Brunsfield: profile, bolt holes, starter mount, dowel holes drilled + reamed. CEED's CO2 lasers can't cut aluminium; SendCutSend can laser it (≤0.75 in, ±0.005 in) if there's no CNC. 1/4 in × 16 × 16 is ~US$67, so 3/4 in is roughly 3×.</t>
+    <t xml:space="preserve">~16 × 16 in blank; thickness from your stack-up (§13). Machined by the shop (work order) or yourself if you get Brunsfield access: profile, bolt holes, starter mount, dowel holes drilled + reamed. CEED's CO2 lasers can't cut aluminium; SendCutSend can laser it (≤0.75 in, ±0.005 in) if there's no CNC. 1/4 in × 16 × 16 is ~US$67, so 3/4 in is roughly 3×.</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.ebay.com/itm/365068559418</t>
@@ -427,7 +427,7 @@
     <t xml:space="preserve">MAKE: vacuum pump block-off plate (only if the pump hits)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aluminium scrap/plate + O-ring, milled at Brunsfield. Only needed if you delete the pump for clearance.</t>
+    <t xml:space="preserve">Aluminium scrap/plate + O-ring, milled by the shop. Only needed if you delete the pump for clearance.</t>
   </si>
   <si>
     <t xml:space="preserve">R14</t>
@@ -439,6 +439,18 @@
     <t xml:space="preserve">~1.6–1.7 L 75W-90 (check the RX-8 manual).</t>
   </si>
   <si>
+    <t xml:space="preserve">R16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Machining labour: uOttawa work-order shop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qty = estimated shop hours for the adapter plate (~4–7 h incl. CAM/setup), CSC adapter (~1.5–2.5 h) and spacers — a rough guess, get a quote. Unit low = Faculty of Science rate $35/h, unit high = uOttawa community rate $90/h (Engineering students pay $90 unless the shop says otherwise). Set N if you can machine it yourself for free.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAD</t>
+  </si>
+  <si>
     <t xml:space="preserve">R15</t>
   </si>
   <si>
@@ -446,9 +458,6 @@
   </si>
   <si>
     <t xml:space="preserve">No off-the-shelf tool fits a VW crank pilot + RX-8 spline.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAD</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal (CAD)</t>
@@ -1255,8 +1264,8 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">'RX-8 BOM'!H28</f>
-        <v>2475.6605</v>
+        <f aca="false">'RX-8 BOM'!H29</f>
+        <v>2792.0605</v>
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">'8HP BOM'!H23</f>
@@ -1268,8 +1277,8 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">'RX-8 BOM'!I28</f>
-        <v>5925.0081</v>
+        <f aca="false">'RX-8 BOM'!I29</f>
+        <v>6738.6081</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">'8HP BOM'!I23</f>
@@ -1283,7 +1292,7 @@
       <c r="B7" s="5"/>
       <c r="C7" s="7" t="n">
         <f aca="false">IF(B5+B6=0,0,(C5+C6)/(B5+B6))</f>
-        <v>2.39849506740452</v>
+        <v>2.11411843655964</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1458,7 +1467,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1875,7 +1884,7 @@
       </c>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
         <v>96</v>
       </c>
@@ -2343,7 +2352,7 @@
       </c>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
         <v>138</v>
       </c>
@@ -2354,24 +2363,24 @@
         <v>140</v>
       </c>
       <c r="D25" s="15" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>141</v>
       </c>
       <c r="F25" s="16" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="G25" s="16" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="H25" s="17" t="n">
         <f aca="false">IF($J25="Y",$D25*$F25*INDEX(Assumptions!$B$4:$B$6,MATCH($E25,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="I25" s="17" t="n">
         <f aca="false">IF($J25="Y",$D25*$G25*INDEX(Assumptions!$B$4:$B$6,MATCH($E25,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>10</v>
+        <v>720</v>
       </c>
       <c r="J25" s="15" t="s">
         <v>64</v>
@@ -2382,26 +2391,42 @@
       <c r="L25" s="14"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="19" t="s">
+      <c r="A26" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="H26" s="20" t="n">
-        <f aca="false">SUM(H5:H25)</f>
-        <v>2190.85</v>
-      </c>
-      <c r="I26" s="20" t="n">
-        <f aca="false">SUM(I5:I25)</f>
-        <v>5243.37</v>
-      </c>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
+      <c r="B26" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <f aca="false">IF($J26="Y",$D26*$F26*INDEX(Assumptions!$B$4:$B$6,MATCH($E26,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <f aca="false">IF($J26="Y",$D26*$G26*INDEX(Assumptions!$B$4:$B$6,MATCH($E26,Assumptions!$A$4:$A$6,0)),0)</f>
+        <v>10</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="K26" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="L26" s="14"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2"/>
@@ -2411,15 +2436,15 @@
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
       <c r="G27" s="19" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H27" s="20" t="n">
-        <f aca="false">H26*Assumptions!$B$8</f>
-        <v>284.8105</v>
+        <f aca="false">SUM(H5:H26)</f>
+        <v>2470.85</v>
       </c>
       <c r="I27" s="20" t="n">
-        <f aca="false">I26*Assumptions!$B$8</f>
-        <v>681.6381</v>
+        <f aca="false">SUM(I5:I26)</f>
+        <v>5963.37</v>
       </c>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
@@ -2432,33 +2457,55 @@
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
-      <c r="G28" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="H28" s="22" t="n">
-        <f aca="false">H26+H27</f>
-        <v>2475.6605</v>
-      </c>
-      <c r="I28" s="22" t="n">
-        <f aca="false">I26+I27</f>
-        <v>5925.0081</v>
+      <c r="G28" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <f aca="false">H27*Assumptions!$B$8</f>
+        <v>321.2105</v>
+      </c>
+      <c r="I28" s="20" t="n">
+        <f aca="false">I27*Assumptions!$B$8</f>
+        <v>775.2381</v>
       </c>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
     </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="H29" s="22" t="n">
+        <f aca="false">H27+H28</f>
+        <v>2792.0605</v>
+      </c>
+      <c r="I29" s="22" t="n">
+        <f aca="false">I27+I28</f>
+        <v>6738.6081</v>
+      </c>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
+      <c r="L29" s="2"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:K25">
+  <conditionalFormatting sqref="A5:K26">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$J5="N"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J25" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J26" type="list">
       <formula1>"Y,N"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E25" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E26" type="list">
       <formula1>"CAD,USD,GBP"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2510,7 +2557,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2594,13 +2641,13 @@
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D5" s="15" t="n">
         <v>1</v>
@@ -2629,18 +2676,18 @@
         <v>65</v>
       </c>
       <c r="L5" s="18" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>1</v>
@@ -2669,18 +2716,18 @@
         <v>95</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D7" s="15" t="n">
         <v>1</v>
@@ -2709,12 +2756,12 @@
         <v>65</v>
       </c>
       <c r="L7" s="18" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>68</v>
@@ -2747,18 +2794,18 @@
         <v>65</v>
       </c>
       <c r="L8" s="18" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>1</v>
@@ -2787,18 +2834,18 @@
         <v>65</v>
       </c>
       <c r="L9" s="18" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>1</v>
@@ -2827,18 +2874,18 @@
         <v>65</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>1</v>
@@ -2867,18 +2914,18 @@
         <v>65</v>
       </c>
       <c r="L11" s="18" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>1</v>
@@ -2907,18 +2954,18 @@
         <v>65</v>
       </c>
       <c r="L12" s="18" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>1</v>
@@ -2947,18 +2994,18 @@
         <v>65</v>
       </c>
       <c r="L13" s="18" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>1</v>
@@ -2990,13 +3037,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D15" s="15" t="n">
         <v>1</v>
@@ -3025,15 +3072,15 @@
         <v>65</v>
       </c>
       <c r="L15" s="18" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="15" t="n">
@@ -3066,13 +3113,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>1</v>
@@ -3101,18 +3148,18 @@
         <v>65</v>
       </c>
       <c r="L17" s="18" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D18" s="15" t="n">
         <v>1</v>
@@ -3141,18 +3188,18 @@
         <v>65</v>
       </c>
       <c r="L18" s="18" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D19" s="15" t="n">
         <v>1</v>
@@ -3184,13 +3231,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D20" s="15" t="n">
         <v>1</v>
@@ -3219,7 +3266,7 @@
         <v>65</v>
       </c>
       <c r="L20" s="18" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3230,7 +3277,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="19" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="H21" s="20" t="n">
         <f aca="false">SUM(H5:H20)</f>
@@ -3252,7 +3299,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="19" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="H22" s="20" t="n">
         <f aca="false">H21*Assumptions!$B$8</f>
@@ -3274,7 +3321,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="21" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H23" s="22" t="n">
         <f aca="false">H21+H22</f>
@@ -3344,7 +3391,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3356,10 +3403,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>59</v>
@@ -3373,7 +3420,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3384,7 +3431,7 @@
         <v>1.42</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3395,7 +3442,7 @@
         <v>1.85</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,13 +3452,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B8" s="25" t="n">
         <v>0.13</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3421,21 +3468,21 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>

</xml_diff>

<commit_message>
RX-8 make route: machine parts in self-serve school shop (no labour)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0175jEiqU2oBgc19VRi9yMgm
</commit_message>
<xml_diff>
--- a/Gearbox_Options.xlsx
+++ b/Gearbox_Options.xlsx
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Adapter</t>
   </si>
   <si>
-    <t xml:space="preserve">Make your own at Brunsfield (material ~US$150–300), or buy the proven £140 plate + £35 bolts from RX8 Gearbox Adapters.</t>
+    <t xml:space="preserve">Make your own on the school CNC (material ~US$150–300), or buy the proven £140 plate + £35 bolts from RX8 Gearbox Adapters.</t>
   </si>
   <si>
     <t xml:space="preserve">$1,250–1,280 DomiWorks kit (plate + billet flywheel + centre guide). Also sold by a Quebec dealer.</t>
@@ -319,7 +319,7 @@
     <t xml:space="preserve">MAKE: adapter plate — 6061-T6 (or MIC-6 cast) plate</t>
   </si>
   <si>
-    <t xml:space="preserve">~16 × 16 in blank; thickness from your stack-up (§13). Machined by the shop (work order) or yourself if you get Brunsfield access: profile, bolt holes, starter mount, dowel holes drilled + reamed. CEED's CO2 lasers can't cut aluminium; SendCutSend can laser it (≤0.75 in, ±0.005 in) if there's no CNC. 1/4 in × 16 × 16 is ~US$67, so 3/4 in is roughly 3×.</t>
+    <t xml:space="preserve">~16 × 16 in blank; thickness from your stack-up (§13). Machined yourself on the school CNC mill (check travel ≥ plate size, ~16 in): profile, bolt holes, starter mount, dowel holes drilled + reamed. CEED's CO2 lasers can't cut aluminium; SendCutSend can laser it (≤0.75 in, ±0.005 in) if there's no CNC. 1/4 in × 16 × 16 is ~US$67, so 3/4 in is roughly 3×.</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.ebay.com/itm/365068559418</t>
@@ -427,7 +427,7 @@
     <t xml:space="preserve">MAKE: vacuum pump block-off plate (only if the pump hits)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aluminium scrap/plate + O-ring, milled by the shop. Only needed if you delete the pump for clearance.</t>
+    <t xml:space="preserve">Aluminium scrap/plate + O-ring, milled yourself. Only needed if you delete the pump for clearance.</t>
   </si>
   <si>
     <t xml:space="preserve">R14</t>
@@ -445,7 +445,7 @@
     <t xml:space="preserve">Machining labour: uOttawa work-order shop</t>
   </si>
   <si>
-    <t xml:space="preserve">Qty = estimated shop hours for the adapter plate (~4–7 h incl. CAM/setup), CSC adapter (~1.5–2.5 h) and spacers — a rough guess, get a quote. Unit low = Faculty of Science rate $35/h, unit high = uOttawa community rate $90/h (Engineering students pay $90 unless the shop says otherwise). Set N if you can machine it yourself for free.</t>
+    <t xml:space="preserve">Qty = estimated shop hours for the adapter plate (~4–7 h incl. CAM/setup), CSC adapter (~1.5–2.5 h) and spacers — a rough guess, get a quote. Unit low = Faculty of Science rate $35/h, unit high = uOttawa community rate $90/h (Engineering students pay $90 unless the shop says otherwise). OFF: you have free self-serve access to a CNC mill, lathe and welding.</t>
   </si>
   <si>
     <t xml:space="preserve">CAD</t>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B5" s="6" t="n">
         <f aca="false">'RX-8 BOM'!H29</f>
-        <v>2792.0605</v>
+        <v>2475.6605</v>
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">'8HP BOM'!H23</f>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">'RX-8 BOM'!I29</f>
-        <v>6738.6081</v>
+        <v>5925.0081</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">'8HP BOM'!I23</f>
@@ -1292,7 +1292,7 @@
       <c r="B7" s="5"/>
       <c r="C7" s="7" t="n">
         <f aca="false">IF(B5+B6=0,0,(C5+C6)/(B5+B6))</f>
-        <v>2.11411843655964</v>
+        <v>2.39849506740452</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2376,14 +2376,14 @@
       </c>
       <c r="H25" s="17" t="n">
         <f aca="false">IF($J25="Y",$D25*$F25*INDEX(Assumptions!$B$4:$B$6,MATCH($E25,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>280</v>
+        <v>0</v>
       </c>
       <c r="I25" s="17" t="n">
         <f aca="false">IF($J25="Y",$D25*$G25*INDEX(Assumptions!$B$4:$B$6,MATCH($E25,Assumptions!$A$4:$A$6,0)),0)</f>
-        <v>720</v>
+        <v>0</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="K25" s="13" t="s">
         <v>95</v>
@@ -2440,11 +2440,11 @@
       </c>
       <c r="H27" s="20" t="n">
         <f aca="false">SUM(H5:H26)</f>
-        <v>2470.85</v>
+        <v>2190.85</v>
       </c>
       <c r="I27" s="20" t="n">
         <f aca="false">SUM(I5:I26)</f>
-        <v>5963.37</v>
+        <v>5243.37</v>
       </c>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
@@ -2462,11 +2462,11 @@
       </c>
       <c r="H28" s="20" t="n">
         <f aca="false">H27*Assumptions!$B$8</f>
-        <v>321.2105</v>
+        <v>284.8105</v>
       </c>
       <c r="I28" s="20" t="n">
         <f aca="false">I27*Assumptions!$B$8</f>
-        <v>775.2381</v>
+        <v>681.6381</v>
       </c>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
@@ -2484,11 +2484,11 @@
       </c>
       <c r="H29" s="22" t="n">
         <f aca="false">H27+H28</f>
-        <v>2792.0605</v>
+        <v>2475.6605</v>
       </c>
       <c r="I29" s="22" t="n">
         <f aca="false">I27+I28</f>
-        <v>6738.6081</v>
+        <v>5925.0081</v>
       </c>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>

</xml_diff>

<commit_message>
Vacuum pump block-off: collar + O-ring design, not a flat plate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0175jEiqU2oBgc19VRi9yMgm
</commit_message>
<xml_diff>
--- a/Gearbox_Options.xlsx
+++ b/Gearbox_Options.xlsx
@@ -427,7 +427,7 @@
     <t xml:space="preserve">MAKE: vacuum pump block-off plate (only if the pump hits)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aluminium scrap/plate + O-ring, milled yourself. Only needed if you delete the pump for clearance.</t>
+    <t xml:space="preserve">Not a flat plate: copy IE's design — flange + a collar that slides into the pump bore to block the pump's oil feed, sealed with an O-ring (no paper gasket). Lathe for the collar/O-ring groove, mill for the bolt holes. Only needed if you delete the pump for clearance.</t>
   </si>
   <si>
     <t xml:space="preserve">R14</t>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
         <v>132</v>
       </c>

</xml_diff>